<commit_message>
Add a golden dataset for Micro-segments & NBA and For Review
One lead + signal workbook of 26 accounts, run the default way (tier A
and B sent from Scoring), where each account is designed for one NBA or
For Review outcome. The answer key comes from the engine and the routing
in demandai-nba.js; the run, queues and decisions in the review script
were clicked through in the prototype. Added to the prospect-to-signal
map.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XiLXGU1oR1hNbNccyNpRo1
</commit_message>
<xml_diff>
--- a/test-data/Prospect_to_Signal_Map.xlsx
+++ b/test-data/Prospect_to_Signal_Map.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Map" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Map'!$A$1:$K$69</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Map'!$A$1:$K$70</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -534,7 +534,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>68 pairings in total.</t>
+          <t>69 pairings in total.</t>
         </is>
       </c>
     </row>
@@ -549,7 +549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K69"/>
+  <dimension ref="A1:K70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3731,12 +3731,12 @@
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>realistic-sets</t>
+          <t>golden-set</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>R1_Smoke_test_small_clean.xlsx</t>
+          <t>Golden_NBA_and_For_Review.xlsx</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
@@ -3746,7 +3746,7 @@
       </c>
       <c r="E63" s="6" t="inlineStr">
         <is>
-          <t>R1_Smoke_test_small_clean.xlsx (same file)</t>
+          <t>Golden_NBA_and_For_Review.xlsx (same file)</t>
         </is>
       </c>
       <c r="F63" s="4" t="inlineStr">
@@ -3761,12 +3761,12 @@
       </c>
       <c r="H63" s="4" t="inlineStr">
         <is>
-          <t>Upload the file as the prospect list, then drop the same file as the signals.</t>
+          <t>Prospecting with the file; Scoring with the saved list and the same file; "Send tier A and B to NBA"; then For Review.</t>
         </is>
       </c>
       <c r="I63" s="4" t="inlineStr">
         <is>
-          <t>R1: "Answer key - summary", "Answer key - accounts"</t>
+          <t>Golden: "Golden - expected totals", "Golden - accounts", "Review script"</t>
         </is>
       </c>
       <c r="J63" s="4" t="n"/>
@@ -3787,7 +3787,7 @@
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>R2_Pilot_list_week_1.xlsx</t>
+          <t>R1_Smoke_test_small_clean.xlsx</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
@@ -3797,7 +3797,7 @@
       </c>
       <c r="E64" s="6" t="inlineStr">
         <is>
-          <t>R2_Pilot_list_week_1.xlsx (same file)</t>
+          <t>R1_Smoke_test_small_clean.xlsx (same file)</t>
         </is>
       </c>
       <c r="F64" s="4" t="inlineStr">
@@ -3817,7 +3817,7 @@
       </c>
       <c r="I64" s="4" t="inlineStr">
         <is>
-          <t>R2: "Answer key - summary", "Answer key - accounts"</t>
+          <t>R1: "Answer key - summary", "Answer key - accounts"</t>
         </is>
       </c>
       <c r="J64" s="4" t="n"/>
@@ -3838,7 +3838,7 @@
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>R3_Large_list_performance.xlsx</t>
+          <t>R2_Pilot_list_week_1.xlsx</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
@@ -3848,7 +3848,7 @@
       </c>
       <c r="E65" s="6" t="inlineStr">
         <is>
-          <t>R3_Large_list_performance.xlsx (same file)</t>
+          <t>R2_Pilot_list_week_1.xlsx (same file)</t>
         </is>
       </c>
       <c r="F65" s="4" t="inlineStr">
@@ -3868,7 +3868,7 @@
       </c>
       <c r="I65" s="4" t="inlineStr">
         <is>
-          <t>R3: "Answer key - summary", "Answer key - accounts"</t>
+          <t>R2: "Answer key - summary", "Answer key - accounts"</t>
         </is>
       </c>
       <c r="J65" s="4" t="n"/>
@@ -3889,7 +3889,7 @@
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>R4_Pilot_list_week_2.xlsx</t>
+          <t>R3_Large_list_performance.xlsx</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
@@ -3899,7 +3899,7 @@
       </c>
       <c r="E66" s="6" t="inlineStr">
         <is>
-          <t>R4_Pilot_list_week_2.xlsx (same file)</t>
+          <t>R3_Large_list_performance.xlsx (same file)</t>
         </is>
       </c>
       <c r="F66" s="4" t="inlineStr">
@@ -3909,7 +3909,7 @@
       </c>
       <c r="G66" s="4" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="H66" s="4" t="inlineStr">
@@ -3919,14 +3919,10 @@
       </c>
       <c r="I66" s="4" t="inlineStr">
         <is>
-          <t>R4: "Answer key - summary", "Answer key - accounts"</t>
-        </is>
-      </c>
-      <c r="J66" s="4" t="inlineStr">
-        <is>
-          <t>Run after R2, once you have decided R2's items in For Review.</t>
-        </is>
-      </c>
+          <t>R3: "Answer key - summary", "Answer key - accounts"</t>
+        </is>
+      </c>
+      <c r="J66" s="4" t="n"/>
       <c r="K66" s="5" t="inlineStr">
         <is>
           <t>Not run</t>
@@ -3944,7 +3940,7 @@
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>R5_Installed_base_existing_customers.xlsx</t>
+          <t>R4_Pilot_list_week_2.xlsx</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
@@ -3954,7 +3950,7 @@
       </c>
       <c r="E67" s="6" t="inlineStr">
         <is>
-          <t>R5_Installed_base_existing_customers.xlsx (same file)</t>
+          <t>R4_Pilot_list_week_2.xlsx (same file)</t>
         </is>
       </c>
       <c r="F67" s="4" t="inlineStr">
@@ -3964,7 +3960,7 @@
       </c>
       <c r="G67" s="4" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="H67" s="4" t="inlineStr">
@@ -3974,10 +3970,14 @@
       </c>
       <c r="I67" s="4" t="inlineStr">
         <is>
-          <t>R5: "Answer key - summary", "Answer key - accounts"</t>
-        </is>
-      </c>
-      <c r="J67" s="4" t="n"/>
+          <t>R4: "Answer key - summary", "Answer key - accounts"</t>
+        </is>
+      </c>
+      <c r="J67" s="4" t="inlineStr">
+        <is>
+          <t>Run after R2, once you have decided R2's items in For Review.</t>
+        </is>
+      </c>
       <c r="K67" s="5" t="inlineStr">
         <is>
           <t>Not run</t>
@@ -3995,7 +3995,7 @@
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>R6_Net_new_marketing_engagement.xlsx</t>
+          <t>R5_Installed_base_existing_customers.xlsx</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
@@ -4005,7 +4005,7 @@
       </c>
       <c r="E68" s="6" t="inlineStr">
         <is>
-          <t>R6_Net_new_marketing_engagement.xlsx (same file)</t>
+          <t>R5_Installed_base_existing_customers.xlsx (same file)</t>
         </is>
       </c>
       <c r="F68" s="4" t="inlineStr">
@@ -4025,7 +4025,7 @@
       </c>
       <c r="I68" s="4" t="inlineStr">
         <is>
-          <t>R6: "Answer key - summary", "Answer key - accounts"</t>
+          <t>R5: "Answer key - summary", "Answer key - accounts"</t>
         </is>
       </c>
       <c r="J68" s="4" t="n"/>
@@ -4046,7 +4046,7 @@
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>R7_CRM_export_format.xlsx</t>
+          <t>R6_Net_new_marketing_engagement.xlsx</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
@@ -4056,7 +4056,7 @@
       </c>
       <c r="E69" s="6" t="inlineStr">
         <is>
-          <t>R7_CRM_export_format.xlsx (same file)</t>
+          <t>R6_Net_new_marketing_engagement.xlsx (same file)</t>
         </is>
       </c>
       <c r="F69" s="4" t="inlineStr">
@@ -4076,7 +4076,7 @@
       </c>
       <c r="I69" s="4" t="inlineStr">
         <is>
-          <t>R7: "Answer key - summary", "Answer key - accounts"</t>
+          <t>R6: "Answer key - summary", "Answer key - accounts"</t>
         </is>
       </c>
       <c r="J69" s="4" t="n"/>
@@ -4086,10 +4086,61 @@
         </is>
       </c>
     </row>
+    <row r="70">
+      <c r="A70" s="4" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t>realistic-sets</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="inlineStr">
+        <is>
+          <t>R7_CRM_export_format.xlsx</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="inlineStr">
+        <is>
+          <t>Lead template</t>
+        </is>
+      </c>
+      <c r="E70" s="6" t="inlineStr">
+        <is>
+          <t>R7_CRM_export_format.xlsx (same file)</t>
+        </is>
+      </c>
+      <c r="F70" s="4" t="inlineStr">
+        <is>
+          <t>Signal template</t>
+        </is>
+      </c>
+      <c r="G70" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="H70" s="4" t="inlineStr">
+        <is>
+          <t>Upload the file as the prospect list, then drop the same file as the signals.</t>
+        </is>
+      </c>
+      <c r="I70" s="4" t="inlineStr">
+        <is>
+          <t>R7: "Answer key - summary", "Answer key - accounts"</t>
+        </is>
+      </c>
+      <c r="J70" s="4" t="n"/>
+      <c r="K70" s="5" t="inlineStr">
+        <is>
+          <t>Not run</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K69"/>
+  <autoFilter ref="A1:K70"/>
   <dataValidations count="1">
-    <dataValidation sqref="K2:K69" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K70" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not run,Pass,Fail,Blocked,Not in scope"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Golden set: separate prospect and signal files
Split the golden workbook into Golden_1_Prospects.xlsx (for Prospecting),
Golden_2_Signals.xlsx (for Account Scoring) and Golden_3_Answer_key.xlsx.
Checked in the prototype with the two files: same segments, routes and
decisions as the answer key.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XiLXGU1oR1hNbNccyNpRo1
</commit_message>
<xml_diff>
--- a/test-data/Prospect_to_Signal_Map.xlsx
+++ b/test-data/Prospect_to_Signal_Map.xlsx
@@ -3736,7 +3736,7 @@
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>Golden_NBA_and_For_Review.xlsx</t>
+          <t>Golden_1_Prospects.xlsx</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
@@ -3744,9 +3744,9 @@
           <t>Lead template</t>
         </is>
       </c>
-      <c r="E63" s="6" t="inlineStr">
-        <is>
-          <t>Golden_NBA_and_For_Review.xlsx (same file)</t>
+      <c r="E63" s="4" t="inlineStr">
+        <is>
+          <t>Golden_2_Signals.xlsx</t>
         </is>
       </c>
       <c r="F63" s="4" t="inlineStr">
@@ -3761,12 +3761,12 @@
       </c>
       <c r="H63" s="4" t="inlineStr">
         <is>
-          <t>Prospecting with the file; Scoring with the saved list and the same file; "Send tier A and B to NBA"; then For Review.</t>
+          <t>Prospecting with Golden_1; Scoring with the saved list and Golden_2; "Send tier A and B to NBA"; then For Review.</t>
         </is>
       </c>
       <c r="I63" s="4" t="inlineStr">
         <is>
-          <t>Golden: "Golden - expected totals", "Golden - accounts", "Review script"</t>
+          <t>Golden_3_Answer_key.xlsx</t>
         </is>
       </c>
       <c r="J63" s="4" t="n"/>

</xml_diff>